<commit_message>
Update chip report site 2026-09-09
</commit_message>
<xml_diff>
--- a/outputs/chip-report/台股盤後籌碼_2026-05-20.xlsx
+++ b/outputs/chip-report/台股盤後籌碼_2026-05-20.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -57,11 +57,17 @@
     </font>
     <font>
       <name val="Microsoft JhengHei"/>
+      <b val="1"/>
+      <color rgb="009f1239"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Microsoft JhengHei"/>
       <color rgb="001f2d3d"/>
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -113,6 +119,16 @@
         <fgColor rgb="00eef7e8"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00fca5a5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00fff1f2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -140,7 +156,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -185,7 +201,16 @@
     <xf numFmtId="0" fontId="2" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -553,7 +578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N114"/>
+  <dimension ref="A1:N132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -582,7 +607,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>本次為 2026-05-20 正式版，已補入 TWSE 與 TAIFEX 官方數據；加權指數當日高低差使用 TWSE MI_5MINS_HIST 官方資料，散戶與微台欄位沿用全市場 OI 減三大法人多空單的原表邏輯回推。</t>
+          <t>本次為 2026-05-20 正式版，已補入 TWSE 與 TAIFEX 官方數據；散戶位階採近45日相對位階（同值取中間排名），並以小台部位 + 微台部位/5 換算等值口數。</t>
         </is>
       </c>
     </row>
@@ -824,7 +849,7 @@
     </row>
     <row r="20">
       <c r="A20" s="6" t="n">
-        <v>471.9599999999991</v>
+        <v>471.96</v>
       </c>
       <c r="B20" s="6" t="n"/>
       <c r="C20" s="6" t="n"/>
@@ -1041,7 +1066,8 @@
       <c r="G39" s="11" t="n"/>
       <c r="I39" s="11" t="inlineStr">
         <is>
-          <t>外資期貨未平倉與結算比</t>
+          <t>【SETTLE DAY】
+外資期貨未平倉與結算比</t>
         </is>
       </c>
       <c r="J39" s="11" t="n"/>
@@ -1059,7 +1085,7 @@
       <c r="F40" s="6" t="n"/>
       <c r="G40" s="6" t="n"/>
       <c r="I40" s="6" t="n">
-        <v>0</v>
+        <v>5874</v>
       </c>
       <c r="J40" s="6" t="n"/>
       <c r="K40" s="6" t="n"/>
@@ -1092,7 +1118,7 @@
       <c r="G42" s="7" t="n"/>
       <c r="I42" s="7" t="inlineStr">
         <is>
-          <t>-42,762.10 - (-42,762) ≈ 0</t>
+          <t>|-42,762.10| - |-36,888| ≈ 5,874；結算日基準 4/15；當日為結算日，本欄改以前次結算日 4/15 為基準。</t>
         </is>
       </c>
       <c r="J42" s="7" t="n"/>
@@ -1198,7 +1224,8 @@
     <row r="51">
       <c r="A51" s="11" t="inlineStr">
         <is>
-          <t>外資(BC)OP未平倉金額與結算比</t>
+          <t>【SETTLE DAY】
+外資(BC)OP未平倉金額與結算比</t>
         </is>
       </c>
       <c r="B51" s="11" t="n"/>
@@ -1220,7 +1247,7 @@
     </row>
     <row r="52">
       <c r="A52" s="6" t="n">
-        <v>0</v>
+        <v>417656</v>
       </c>
       <c r="B52" s="6" t="n"/>
       <c r="C52" s="6" t="n"/>
@@ -1249,7 +1276,7 @@
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>1,224,012 - 1,224,012(5/20結算日 BC 原始金額)</t>
+          <t>1,224,012 - 806,356(4/15結算日 BC 原始金額)；當日為結算日，本欄改以前次結算日 4/15 為基準。</t>
         </is>
       </c>
       <c r="B54" s="7" t="n"/>
@@ -1283,7 +1310,8 @@
     <row r="57">
       <c r="A57" s="11" t="inlineStr">
         <is>
-          <t>外資(BP)OP未平倉金額與結算比</t>
+          <t>【SETTLE DAY】
+外資(BP)OP未平倉金額與結算比</t>
         </is>
       </c>
       <c r="B57" s="11" t="n"/>
@@ -1305,7 +1333,7 @@
     </row>
     <row r="58" ht="22" customHeight="1">
       <c r="A58" s="6" t="n">
-        <v>0</v>
+        <v>281727</v>
       </c>
       <c r="B58" s="6" t="n"/>
       <c r="C58" s="6" t="n"/>
@@ -1334,7 +1362,7 @@
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
         <is>
-          <t>407,759 - 407,759(5/20結算日 BP 原始金額)</t>
+          <t>407,759 - 126,032(4/15結算日 BP 原始金額)；當日為結算日，本欄改以前次結算日 4/15 為基準。</t>
         </is>
       </c>
       <c r="B60" s="7" t="n"/>
@@ -1487,7 +1515,8 @@
       <c r="G71" s="13" t="n"/>
       <c r="I71" s="13" t="inlineStr">
         <is>
-          <t>自營(BC)OP未平倉金額與結算比</t>
+          <t>【SETTLE DAY】
+自營(BC)OP未平倉金額與結算比</t>
         </is>
       </c>
       <c r="J71" s="13" t="n"/>
@@ -1505,7 +1534,7 @@
       <c r="F72" s="6" t="n"/>
       <c r="G72" s="6" t="n"/>
       <c r="I72" s="6" t="n">
-        <v>0</v>
+        <v>-151637</v>
       </c>
       <c r="J72" s="6" t="n"/>
       <c r="K72" s="6" t="n"/>
@@ -1538,7 +1567,7 @@
       <c r="G74" s="7" t="n"/>
       <c r="I74" s="7" t="inlineStr">
         <is>
-          <t>1,019,525 - 1,019,525(5/20結算日 BC 原始金額)</t>
+          <t>1,019,525 - 1,171,162(4/15結算日 BC 原始金額)；當日為結算日，本欄改以前次結算日 4/15 為基準。</t>
         </is>
       </c>
       <c r="J74" s="7" t="n"/>
@@ -1572,7 +1601,8 @@
       <c r="G77" s="13" t="n"/>
       <c r="I77" s="13" t="inlineStr">
         <is>
-          <t>自營(BP)OP未平倉金額與結算比</t>
+          <t>【SETTLE DAY】
+自營(BP)OP未平倉金額與結算比</t>
         </is>
       </c>
       <c r="J77" s="13" t="n"/>
@@ -1590,7 +1620,7 @@
       <c r="F78" s="6" t="n"/>
       <c r="G78" s="6" t="n"/>
       <c r="I78" s="6" t="n">
-        <v>0</v>
+        <v>91879</v>
       </c>
       <c r="J78" s="6" t="n"/>
       <c r="K78" s="6" t="n"/>
@@ -1623,7 +1653,7 @@
       <c r="G80" s="7" t="n"/>
       <c r="I80" s="7" t="inlineStr">
         <is>
-          <t>357,698 - 357,698(5/20結算日 BP 原始金額)</t>
+          <t>357,698 - 265,819(4/15結算日 BP 原始金額)；當日為結算日，本欄改以前次結算日 4/15 為基準。</t>
         </is>
       </c>
       <c r="J80" s="7" t="n"/>
@@ -1720,12 +1750,12 @@
     </row>
     <row r="92">
       <c r="A92" s="6" t="n">
-        <v>35380</v>
+        <v>24439</v>
       </c>
       <c r="B92" s="6" t="n"/>
       <c r="C92" s="6" t="n"/>
       <c r="E92" s="6" t="n">
-        <v>26740</v>
+        <v>15799</v>
       </c>
       <c r="F92" s="6" t="n"/>
       <c r="G92" s="6" t="n"/>
@@ -1749,14 +1779,14 @@
     <row r="94">
       <c r="A94" s="7" t="inlineStr">
         <is>
-          <t>MTX 全市場OI 40,329 - (自營1,737 + 投信103 + 外資3,109)</t>
+          <t>MTX 全市場OI 29,388 - (自營1,737 + 投信103 + 外資3,109)</t>
         </is>
       </c>
       <c r="B94" s="7" t="n"/>
       <c r="C94" s="7" t="n"/>
       <c r="E94" s="7" t="inlineStr">
         <is>
-          <t>MTX 全市場OI 40,329 - (自營10,339 + 投信103 + 外資3,147)</t>
+          <t>MTX 全市場OI 29,388 - (自營10,339 + 投信103 + 外資3,147)</t>
         </is>
       </c>
       <c r="F94" s="7" t="n"/>
@@ -1811,12 +1841,12 @@
       <c r="B98" s="6" t="n"/>
       <c r="C98" s="6" t="n"/>
       <c r="E98" s="6" t="n">
-        <v>66120</v>
+        <v>50616</v>
       </c>
       <c r="F98" s="6" t="n"/>
       <c r="G98" s="6" t="n"/>
       <c r="I98" s="6" t="n">
-        <v>36497</v>
+        <v>20993</v>
       </c>
       <c r="J98" s="6" t="n"/>
       <c r="K98" s="6" t="n"/>
@@ -1835,21 +1865,21 @@
     <row r="100">
       <c r="A100" s="7" t="inlineStr">
         <is>
-          <t>35,380 - 26,740</t>
+          <t>24,439 - 15,799</t>
         </is>
       </c>
       <c r="B100" s="7" t="n"/>
       <c r="C100" s="7" t="n"/>
       <c r="E100" s="7" t="inlineStr">
         <is>
-          <t>TMF 全市場OI 68,655 - (自營1,915 + 投信0 + 外資620)</t>
+          <t>TMF 全市場OI 53,151 - (自營1,915 + 投信0 + 外資620)</t>
         </is>
       </c>
       <c r="F100" s="7" t="n"/>
       <c r="G100" s="7" t="n"/>
       <c r="I100" s="7" t="inlineStr">
         <is>
-          <t>TMF 全市場OI 68,655 - (自營31,366 + 投信0 + 外資792)</t>
+          <t>TMF 全市場OI 53,151 - (自營31,366 + 投信0 + 外資792)</t>
         </is>
       </c>
       <c r="J100" s="7" t="n"/>
@@ -1881,10 +1911,17 @@
       </c>
       <c r="F103" s="15" t="n"/>
       <c r="G103" s="15" t="n"/>
+      <c r="I103" s="15" t="inlineStr">
+        <is>
+          <t>小台+微台等值多單</t>
+        </is>
+      </c>
+      <c r="J103" s="15" t="n"/>
+      <c r="K103" s="15" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="6" t="n">
-        <v>43.14762216881509</v>
+        <v>55.73366446539105</v>
       </c>
       <c r="B104" s="6" t="n"/>
       <c r="C104" s="6" t="n"/>
@@ -1893,6 +1930,11 @@
       </c>
       <c r="F104" s="6" t="n"/>
       <c r="G104" s="6" t="n"/>
+      <c r="I104" s="6" t="n">
+        <v>34562.2</v>
+      </c>
+      <c r="J104" s="6" t="n"/>
+      <c r="K104" s="6" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="6" t="n"/>
@@ -1901,22 +1943,32 @@
       <c r="E105" s="6" t="n"/>
       <c r="F105" s="6" t="n"/>
       <c r="G105" s="6" t="n"/>
+      <c r="I105" s="6" t="n"/>
+      <c r="J105" s="6" t="n"/>
+      <c r="K105" s="6" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="7" t="inlineStr">
         <is>
-          <t>(29,623 / 68,655) x 100</t>
+          <t>(29,623 / 53,151) x 100</t>
         </is>
       </c>
       <c r="B106" s="7" t="n"/>
       <c r="C106" s="7" t="n"/>
       <c r="E106" s="7" t="inlineStr">
         <is>
-          <t>66,120 - 36,497</t>
+          <t>50,616 - 20,993</t>
         </is>
       </c>
       <c r="F106" s="7" t="n"/>
       <c r="G106" s="7" t="n"/>
+      <c r="I106" s="7" t="inlineStr">
+        <is>
+          <t>24,439 + 50,616 / 5；微台 5 口換算 1 口小台等值</t>
+        </is>
+      </c>
+      <c r="J106" s="7" t="n"/>
+      <c r="K106" s="7" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="7" t="n"/>
@@ -1925,23 +1977,262 @@
       <c r="E107" s="7" t="n"/>
       <c r="F107" s="7" t="n"/>
       <c r="G107" s="7" t="n"/>
+      <c r="I107" s="7" t="n"/>
+      <c r="J107" s="7" t="n"/>
+      <c r="K107" s="7" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="15" t="inlineStr">
+        <is>
+          <t>小台+微台等值空單</t>
+        </is>
+      </c>
+      <c r="B109" s="15" t="n"/>
+      <c r="C109" s="15" t="n"/>
+      <c r="E109" s="15" t="inlineStr">
+        <is>
+          <t>小台+微台等值淨多空</t>
+        </is>
+      </c>
+      <c r="F109" s="15" t="n"/>
+      <c r="G109" s="15" t="n"/>
+      <c r="I109" s="15" t="inlineStr">
+        <is>
+          <t>散戶多方位階(45日)</t>
+        </is>
+      </c>
+      <c r="J109" s="15" t="n"/>
+      <c r="K109" s="15" t="n"/>
     </row>
     <row r="110">
-      <c r="A110" s="16" t="inlineStr">
-        <is>
-          <t>這是 2026-05-20 的盤後籌碼正式版：加權指數收 40,020.82 點、跌 154.74 點，盤中最高 40,439.04 點、最低 39,967.08 點，成交值約 10,275.53 億元；TWSE 信用交易統計已補回，融資金額餘額 5,020.79 億、較前一交易日增加 51.92 億，融券餘額 244,522 張、較前一交易日增加 5,317 張。TAIFEX 的外資(大小台)期貨未平倉依原表合併口徑 = TXF + MXF/4 + TMF/20，5/20 約為 -42,762，與結算比約 0、與前日增減約 1,822；主表 OP 欄位維持 BC-SC 與 BP-SP 的淨額口徑。</t>
-        </is>
-      </c>
-    </row>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
+      <c r="A110" s="6" t="n">
+        <v>19997.6</v>
+      </c>
+      <c r="B110" s="6" t="n"/>
+      <c r="C110" s="6" t="n"/>
+      <c r="E110" s="6" t="n">
+        <v>14564.6</v>
+      </c>
+      <c r="F110" s="6" t="n"/>
+      <c r="G110" s="6" t="n"/>
+      <c r="I110" s="6" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="J110" s="6" t="n"/>
+      <c r="K110" s="6" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="6" t="n"/>
+      <c r="B111" s="6" t="n"/>
+      <c r="C111" s="6" t="n"/>
+      <c r="E111" s="6" t="n"/>
+      <c r="F111" s="6" t="n"/>
+      <c r="G111" s="6" t="n"/>
+      <c r="I111" s="6" t="n"/>
+      <c r="J111" s="6" t="n"/>
+      <c r="K111" s="6" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="7" t="inlineStr">
+        <is>
+          <t>15,799 + 20,993 / 5；微台 5 口換算 1 口小台等值</t>
+        </is>
+      </c>
+      <c r="B112" s="7" t="n"/>
+      <c r="C112" s="7" t="n"/>
+      <c r="E112" s="7" t="inlineStr">
+        <is>
+          <t>34,562.2 - 19,997.6</t>
+        </is>
+      </c>
+      <c r="F112" s="7" t="n"/>
+      <c r="G112" s="7" t="n"/>
+      <c r="I112" s="7" t="inlineStr">
+        <is>
+          <t>近45日相對位階（同值取中間排名）= (低於本日筆數 + 同值筆數 / 2) / 樣本數 x 100。 小台＋微台等值口數；微台 5 口換算為 1 口小台等值。；目前樣本 20 筆。</t>
+        </is>
+      </c>
+      <c r="J112" s="7" t="n"/>
+      <c r="K112" s="7" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="7" t="n"/>
+      <c r="B113" s="7" t="n"/>
+      <c r="C113" s="7" t="n"/>
+      <c r="E113" s="7" t="n"/>
+      <c r="F113" s="7" t="n"/>
+      <c r="G113" s="7" t="n"/>
+      <c r="I113" s="7" t="n"/>
+      <c r="J113" s="7" t="n"/>
+      <c r="K113" s="7" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="15" t="inlineStr">
+        <is>
+          <t>散戶空方位階(45日)</t>
+        </is>
+      </c>
+      <c r="B115" s="15" t="n"/>
+      <c r="C115" s="15" t="n"/>
+      <c r="E115" s="16" t="inlineStr">
+        <is>
+          <t>【CROWDING】
+散戶淨多空位階(45日)</t>
+        </is>
+      </c>
+      <c r="F115" s="16" t="n"/>
+      <c r="G115" s="16" t="n"/>
+      <c r="I115" s="16" t="inlineStr">
+        <is>
+          <t>【CROWDING】
+散戶多單持倉占比位階(45日)</t>
+        </is>
+      </c>
+      <c r="J115" s="16" t="n"/>
+      <c r="K115" s="16" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="6" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="B116" s="6" t="n"/>
+      <c r="C116" s="6" t="n"/>
+      <c r="E116" s="17" t="n">
+        <v>92.5</v>
+      </c>
+      <c r="F116" s="17" t="n"/>
+      <c r="G116" s="17" t="n"/>
+      <c r="I116" s="17" t="n">
+        <v>97.5</v>
+      </c>
+      <c r="J116" s="17" t="n"/>
+      <c r="K116" s="17" t="n"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="6" t="n"/>
+      <c r="B117" s="6" t="n"/>
+      <c r="C117" s="6" t="n"/>
+      <c r="E117" s="17" t="n"/>
+      <c r="F117" s="17" t="n"/>
+      <c r="G117" s="17" t="n"/>
+      <c r="I117" s="17" t="n"/>
+      <c r="J117" s="17" t="n"/>
+      <c r="K117" s="17" t="n"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="7" t="inlineStr">
+        <is>
+          <t>近45日相對位階（同值取中間排名）= (低於本日筆數 + 同值筆數 / 2) / 樣本數 x 100。 小台＋微台等值口數；微台 5 口換算為 1 口小台等值。；目前樣本 20 筆。</t>
+        </is>
+      </c>
+      <c r="B118" s="7" t="n"/>
+      <c r="C118" s="7" t="n"/>
+      <c r="E118" s="18" t="inlineStr">
+        <is>
+          <t>近45日相對位階（同值取中間排名）= (低於本日筆數 + 同值筆數 / 2) / 樣本數 x 100。 小台＋微台等值口數；微台 5 口換算為 1 口小台等值。；目前樣本 20 筆。</t>
+        </is>
+      </c>
+      <c r="F118" s="18" t="n"/>
+      <c r="G118" s="18" t="n"/>
+      <c r="I118" s="18" t="inlineStr">
+        <is>
+          <t>近45日相對位階（同值取中間排名）= (低於本日筆數 + 同值筆數 / 2) / 樣本數 x 100。 小台＋微台等值口數；微台 5 口換算為 1 口小台等值。；目前樣本 20 筆。</t>
+        </is>
+      </c>
+      <c r="J118" s="18" t="n"/>
+      <c r="K118" s="18" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="7" t="n"/>
+      <c r="B119" s="7" t="n"/>
+      <c r="C119" s="7" t="n"/>
+      <c r="E119" s="18" t="n"/>
+      <c r="F119" s="18" t="n"/>
+      <c r="G119" s="18" t="n"/>
+      <c r="I119" s="18" t="n"/>
+      <c r="J119" s="18" t="n"/>
+      <c r="K119" s="18" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="15" t="inlineStr">
+        <is>
+          <t>散戶空單持倉占比位階(45日)</t>
+        </is>
+      </c>
+      <c r="B121" s="15" t="n"/>
+      <c r="C121" s="15" t="n"/>
+      <c r="E121" s="16" t="inlineStr">
+        <is>
+          <t>【CROWDING】
+微台多空比位階(45日)</t>
+        </is>
+      </c>
+      <c r="F121" s="16" t="n"/>
+      <c r="G121" s="16" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="6" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="B122" s="6" t="n"/>
+      <c r="C122" s="6" t="n"/>
+      <c r="E122" s="17" t="n">
+        <v>92.5</v>
+      </c>
+      <c r="F122" s="17" t="n"/>
+      <c r="G122" s="17" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="6" t="n"/>
+      <c r="B123" s="6" t="n"/>
+      <c r="C123" s="6" t="n"/>
+      <c r="E123" s="17" t="n"/>
+      <c r="F123" s="17" t="n"/>
+      <c r="G123" s="17" t="n"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="7" t="inlineStr">
+        <is>
+          <t>近45日相對位階（同值取中間排名）= (低於本日筆數 + 同值筆數 / 2) / 樣本數 x 100。 小台＋微台等值口數；微台 5 口換算為 1 口小台等值。；目前樣本 20 筆。</t>
+        </is>
+      </c>
+      <c r="B124" s="7" t="n"/>
+      <c r="C124" s="7" t="n"/>
+      <c r="E124" s="18" t="inlineStr">
+        <is>
+          <t>近45日相對位階（同值取中間排名）= (低於本日筆數 + 同值筆數 / 2) / 樣本數 x 100。 小台＋微台等值口數；微台 5 口換算為 1 口小台等值。；目前樣本 20 筆。</t>
+        </is>
+      </c>
+      <c r="F124" s="18" t="n"/>
+      <c r="G124" s="18" t="n"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="7" t="n"/>
+      <c r="B125" s="7" t="n"/>
+      <c r="C125" s="7" t="n"/>
+      <c r="E125" s="18" t="n"/>
+      <c r="F125" s="18" t="n"/>
+      <c r="G125" s="18" t="n"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="19" t="inlineStr">
+        <is>
+          <t>這是 2026-05-20 的盤後籌碼正式版：加權指數收 40,020.82 點、跌 154.74 點，盤中最高 40,439.04 點、最低 39,967.08 點，成交值約 10,275.53 億元；TWSE 信用交易統計已補回，融資金額餘額 5,020.79 億、較前一交易日增加 51.92 億，融券餘額 244,522 張、較前一交易日增加 5,317 張。TAIFEX 的外資(大小台)期貨未平倉依原表合併口徑 = TXF + MXF/4 + TMF/20，5/20 約為 -42,762，與結算比約 5,874、與前日增減約 1,822；主表 OP 欄位維持 BC-SC 與 BP-SP 的淨額口徑。</t>
+        </is>
+      </c>
+    </row>
+    <row r="129"/>
+    <row r="130"/>
+    <row r="131"/>
+    <row r="132"/>
   </sheetData>
-  <mergeCells count="137">
+  <mergeCells count="164">
+    <mergeCell ref="E116:G117"/>
+    <mergeCell ref="I103:K103"/>
     <mergeCell ref="E13:G13"/>
     <mergeCell ref="E72:G73"/>
     <mergeCell ref="I97:K97"/>
+    <mergeCell ref="I110:K111"/>
     <mergeCell ref="A34:C35"/>
     <mergeCell ref="A57:C57"/>
     <mergeCell ref="A71:C71"/>
@@ -1953,12 +2244,16 @@
     <mergeCell ref="E57:G57"/>
     <mergeCell ref="E48:G49"/>
     <mergeCell ref="A91:C91"/>
+    <mergeCell ref="I104:K105"/>
+    <mergeCell ref="A128:N132"/>
     <mergeCell ref="A16:C17"/>
     <mergeCell ref="I26:K27"/>
+    <mergeCell ref="I106:K107"/>
     <mergeCell ref="I65:K65"/>
     <mergeCell ref="A77:C77"/>
     <mergeCell ref="E74:G75"/>
     <mergeCell ref="A83:C83"/>
+    <mergeCell ref="E121:G121"/>
     <mergeCell ref="I68:K69"/>
     <mergeCell ref="A86:C87"/>
     <mergeCell ref="I58:K59"/>
@@ -1966,9 +2261,11 @@
     <mergeCell ref="A22:C23"/>
     <mergeCell ref="I42:K43"/>
     <mergeCell ref="I20:K21"/>
+    <mergeCell ref="A116:C117"/>
     <mergeCell ref="I60:K61"/>
     <mergeCell ref="A20:C21"/>
     <mergeCell ref="A72:C73"/>
+    <mergeCell ref="I115:K115"/>
     <mergeCell ref="E100:G101"/>
     <mergeCell ref="A28:C29"/>
     <mergeCell ref="A1:N1"/>
@@ -1976,11 +2273,13 @@
     <mergeCell ref="E22:G23"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="E14:G15"/>
+    <mergeCell ref="A110:C111"/>
     <mergeCell ref="A48:C49"/>
     <mergeCell ref="A97:C97"/>
+    <mergeCell ref="E122:G123"/>
     <mergeCell ref="E78:G79"/>
-    <mergeCell ref="A110:N114"/>
     <mergeCell ref="I51:K51"/>
+    <mergeCell ref="A121:C121"/>
     <mergeCell ref="A54:C55"/>
     <mergeCell ref="I72:K73"/>
     <mergeCell ref="A13:C13"/>
@@ -1988,10 +2287,12 @@
     <mergeCell ref="E97:G97"/>
     <mergeCell ref="A12:N12"/>
     <mergeCell ref="A31:C31"/>
+    <mergeCell ref="E109:G109"/>
     <mergeCell ref="A74:C75"/>
     <mergeCell ref="A46:C47"/>
     <mergeCell ref="A51:C51"/>
     <mergeCell ref="E71:G71"/>
+    <mergeCell ref="I112:K113"/>
     <mergeCell ref="E46:G47"/>
     <mergeCell ref="E40:G41"/>
     <mergeCell ref="A4:N4"/>
@@ -2007,6 +2308,7 @@
     <mergeCell ref="E26:G27"/>
     <mergeCell ref="A68:C69"/>
     <mergeCell ref="E66:G67"/>
+    <mergeCell ref="E124:G125"/>
     <mergeCell ref="E106:G107"/>
     <mergeCell ref="E65:G65"/>
     <mergeCell ref="A52:C53"/>
@@ -2024,10 +2326,15 @@
     <mergeCell ref="A78:C79"/>
     <mergeCell ref="E60:G61"/>
     <mergeCell ref="A6:C7"/>
+    <mergeCell ref="I109:K109"/>
+    <mergeCell ref="I116:K117"/>
+    <mergeCell ref="E115:G115"/>
     <mergeCell ref="I13:K13"/>
     <mergeCell ref="A80:C81"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="I100:K101"/>
+    <mergeCell ref="E118:G119"/>
+    <mergeCell ref="I118:K119"/>
     <mergeCell ref="E28:G29"/>
     <mergeCell ref="E94:G95"/>
     <mergeCell ref="A26:C27"/>
@@ -2035,30 +2342,37 @@
     <mergeCell ref="I57:K57"/>
     <mergeCell ref="I48:K49"/>
     <mergeCell ref="A104:C105"/>
+    <mergeCell ref="A122:C123"/>
     <mergeCell ref="E80:G81"/>
     <mergeCell ref="E51:G51"/>
     <mergeCell ref="E16:G17"/>
     <mergeCell ref="I94:K95"/>
+    <mergeCell ref="A112:C113"/>
     <mergeCell ref="A106:C107"/>
     <mergeCell ref="A64:N64"/>
     <mergeCell ref="I71:K71"/>
     <mergeCell ref="I74:K75"/>
+    <mergeCell ref="E112:G113"/>
     <mergeCell ref="A58:C59"/>
     <mergeCell ref="I80:K81"/>
     <mergeCell ref="A40:C41"/>
     <mergeCell ref="A98:C99"/>
     <mergeCell ref="A90:N90"/>
     <mergeCell ref="A60:C61"/>
+    <mergeCell ref="A109:C109"/>
     <mergeCell ref="I66:K67"/>
     <mergeCell ref="E91:G91"/>
     <mergeCell ref="E25:G25"/>
     <mergeCell ref="E98:G99"/>
     <mergeCell ref="E20:G21"/>
     <mergeCell ref="I19:K19"/>
+    <mergeCell ref="A115:C115"/>
     <mergeCell ref="A19:C19"/>
     <mergeCell ref="A66:C67"/>
+    <mergeCell ref="A124:C125"/>
     <mergeCell ref="I22:K23"/>
     <mergeCell ref="I28:K29"/>
+    <mergeCell ref="A118:C119"/>
     <mergeCell ref="A39:C39"/>
     <mergeCell ref="I52:K53"/>
     <mergeCell ref="I92:K93"/>
@@ -2071,6 +2385,7 @@
     <mergeCell ref="A32:C33"/>
     <mergeCell ref="E39:G39"/>
     <mergeCell ref="A14:C15"/>
+    <mergeCell ref="E110:G111"/>
     <mergeCell ref="A42:C43"/>
     <mergeCell ref="A100:C101"/>
     <mergeCell ref="A65:C65"/>

</xml_diff>